<commit_message>
chore(vérification) : vérifier le backlog + planif + maquette + routes/actions http avec le prof
[25][Done]
</commit_message>
<xml_diff>
--- a/doc/analyse_verbesHTTP.xlsx
+++ b/doc/analyse_verbesHTTP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe40boh\Documents\Github\P_Web_294-Passion_lecture-Vue.js\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47AA86EE-7C54-4C94-84DE-9AA4E79F13E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C5C4CE-1EB6-4692-B9BC-475B3150AD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
   <si>
     <t>Action</t>
   </si>
@@ -54,9 +54,6 @@
     <t>POST</t>
   </si>
   <si>
-    <t>/api/books/add</t>
-  </si>
-  <si>
     <t>oui</t>
   </si>
   <si>
@@ -66,18 +63,12 @@
     <t>PUT</t>
   </si>
   <si>
-    <t>/api/books/:id/modify</t>
-  </si>
-  <si>
     <t>Supprimer un livre</t>
   </si>
   <si>
     <t>DELETE</t>
   </si>
   <si>
-    <t>/api/books/:id/delete</t>
-  </si>
-  <si>
     <t>Récupérer les détails d'un livres</t>
   </si>
   <si>
@@ -90,25 +81,28 @@
     <t>Récupérer les 5 premiers livres</t>
   </si>
   <si>
-    <t>/api</t>
-  </si>
-  <si>
     <t>Ajouter un commentaire</t>
   </si>
   <si>
-    <t>/api/books/:id/comments/add</t>
-  </si>
-  <si>
     <t>Modifier un commentaire</t>
   </si>
   <si>
-    <t>/api/comments/:id/modify</t>
-  </si>
-  <si>
     <t>Supprimer un commentaire</t>
   </si>
   <si>
-    <t>/api/comments/:id/delete</t>
+    <t>/api/books?limit=5</t>
+  </si>
+  <si>
+    <t>/api/books/:id/comments</t>
+  </si>
+  <si>
+    <t>/api/books/:id/comments/:comment_id</t>
+  </si>
+  <si>
+    <t>tous les livres d'un user</t>
+  </si>
+  <si>
+    <t>tous les livres d'une catégorie</t>
   </si>
 </sst>
 </file>
@@ -164,8 +158,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F94B418-7A92-4C28-AED0-625210A1363D}" name="Tableau1" displayName="Tableau1" ref="A1:D10" totalsRowShown="0">
-  <autoFilter ref="A1:D10" xr:uid="{2F94B418-7A92-4C28-AED0-625210A1363D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F94B418-7A92-4C28-AED0-625210A1363D}" name="Tableau1" displayName="Tableau1" ref="A1:D12" totalsRowShown="0">
+  <autoFilter ref="A1:D12" xr:uid="{2F94B418-7A92-4C28-AED0-625210A1363D}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{AA191AA4-87E2-4EF4-9C7C-C6EB869CA045}" name="Action"/>
     <tableColumn id="2" xr3:uid="{BE2F96E2-7998-4C9C-9CDC-AC83C7B51B3D}" name="Verbe"/>
@@ -439,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="35.7109375" customWidth="1"/>
@@ -461,7 +455,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -475,7 +469,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -489,13 +483,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -509,63 +503,63 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
         <v>9</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
         <v>11</v>
       </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
         <v>15</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
       </c>
       <c r="D9" t="s">
         <v>6</v>
@@ -573,16 +567,26 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
doc(analyse des routes) : réviser le document en se basant sur les conseils du prof
[15][Done]
</commit_message>
<xml_diff>
--- a/doc/analyse_verbesHTTP.xlsx
+++ b/doc/analyse_verbesHTTP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe40boh\Documents\Github\P_Web_294-Passion_lecture-Vue.js\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C5C4CE-1EB6-4692-B9BC-475B3150AD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B452E2F-7C83-4995-8FAA-D6D13553C333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="28">
   <si>
     <t>Action</t>
   </si>
@@ -72,9 +72,6 @@
     <t>Récupérer les détails d'un livres</t>
   </si>
   <si>
-    <t>/api/books/:id</t>
-  </si>
-  <si>
     <t>Récupérer tous les livres et catégories</t>
   </si>
   <si>
@@ -93,16 +90,25 @@
     <t>/api/books?limit=5</t>
   </si>
   <si>
-    <t>/api/books/:id/comments</t>
-  </si>
-  <si>
-    <t>/api/books/:id/comments/:comment_id</t>
-  </si>
-  <si>
-    <t>tous les livres d'un user</t>
-  </si>
-  <si>
-    <t>tous les livres d'une catégorie</t>
+    <t>Récupérer tous les livres d'un user</t>
+  </si>
+  <si>
+    <t>Récupérer tous les livres d'une catégorie</t>
+  </si>
+  <si>
+    <t>/api/users/:user_id/books</t>
+  </si>
+  <si>
+    <t>/api/books/categorie/:categorie_id</t>
+  </si>
+  <si>
+    <t>/api/books/:book_id</t>
+  </si>
+  <si>
+    <t>/api/books/:book_id/comments</t>
+  </si>
+  <si>
+    <t>/api/books/:book_id/comments/:comment_id</t>
   </si>
 </sst>
 </file>
@@ -436,7 +442,7 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="35.7109375" customWidth="1"/>
+    <col min="1" max="4" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -455,13 +461,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -469,7 +475,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -489,7 +495,7 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -497,41 +503,41 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -539,13 +545,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
         <v>9</v>
@@ -553,40 +559,58 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>